<commit_message>
Switched to Global Priority Queue, added Source URL Tracking and added Crawl Reports
</commit_message>
<xml_diff>
--- a/emails.xlsx
+++ b/emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A310"/>
+  <dimension ref="A1:B303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -422,2167 +422,3633 @@
           <t>Email</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>aamenazaidi@csjmu.ac.in</t>
+          <t>aayushi@hum.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>abhilashasharma23@csjmu.ac.in</t>
+          <t>abdeoghare@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>abhishek@csjmu.ac.in</t>
+          <t>abhijeet@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>abhishekchandra@csjmu.ac.in</t>
+          <t>abhishek@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>abhishekdwivedi778@csjmu.ac.in</t>
+          <t>adey6601@gmail.com</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>abhishekdwivedi@csjmu.ac.in</t>
+          <t>agnibis@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>abhishekmishra@csjmu.ac.in</t>
+          <t>ajitesh@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>abhishektiwari@csjmu.ac.in</t>
+          <t>akarim@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>adarshkumarsrivastava@csjmu.ac.in</t>
+          <t>akdey@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ahmadabdullah@csjmu.ac.in</t>
+          <t>alfabisoi@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>aishwaryaarya@csjmu.ac.in</t>
+          <t>alokmeher6820@gmail.com</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ajay@csjmu.ac.in</t>
+          <t>amarjeetkumar9577@gmail.com</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ajaykp4@csjmu.ac.in</t>
+          <t>ambika@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ajaykumar@csjmu.ac.in</t>
+          <t>ambrish@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ajaykumargupta@csjmu.ac.in</t>
+          <t>aminul@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ajaypratapsingh@csjmu.ac.in</t>
+          <t>amitkdas@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ajaytiwari@csjmu.ac.in</t>
+          <t>amritesh@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ajeetsrivastava@csjmu.ac.in</t>
+          <t>anishkumarsaha@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>akankshabajpai@csjmu.ac.in</t>
+          <t>ankush@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>akaty@csjmu.ac.in</t>
+          <t>anup@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>akhileshsingh@csjmu.ac.in</t>
+          <t>anupam@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>akhlendrapratap@csjmu.ac.in</t>
+          <t>aparajita.dutta@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>alkagupta@csjmu.ac.in</t>
+          <t>aparna_st@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>alok@csjmu.ac.in</t>
+          <t>arif@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>alokpandey@csjmu.ac.in</t>
+          <t>arijit@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>alokshukla51@rediffmail.com</t>
+          <t>arjun@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>amanrathaur@csjmu.ac.in</t>
+          <t>arnab@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>amitkatiyar@csjmu.ac.in</t>
+          <t>arun@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>amitvirmani@csjmu.ac.in</t>
+          <t>arun@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>amritasingh@csjmu.ac.in</t>
+          <t>arup@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>anamikadixit@csjmu.ac.in</t>
+          <t>arupgoswami@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>anandgupta@csjmu.ac.in</t>
+          <t>aryaman@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>anitaawasthi@csjmu.ac.in</t>
+          <t>asharani@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>anjudixit@csjmu.ac.in</t>
+          <t>ashim@mba.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>anjusingh@csjmu.ac.in</t>
+          <t>ashish@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ankit@csjmu.ac.in</t>
+          <t>ashraf@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ankitkumar@csjmu.ac.in</t>
+          <t>asim@phy.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>annikasingh@csjmu.ac.in</t>
+          <t>atanu@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>anshu@csjmu.ac.in</t>
+          <t>avadh@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>anshuyadav@csjmu.ac.in</t>
+          <t>avijit@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>anukalani@csjmu.ac.in</t>
+          <t>avishekray@hum.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>anupmayadav@csjmu.ac.in</t>
+          <t>badal@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>anupriyakapoor@csjmu.ac.in</t>
+          <t>banani@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>aparnakatiyar@csjmu.ac.in</t>
+          <t>barun@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>apsingh@csjmu.ac.in</t>
+          <t>bbhowmick@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>arajendiran@csjmu.ac.in</t>
+          <t>bdey@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>arpit@csjmu.ac.in</t>
+          <t>bganguly@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>arpitasingh@csjmu.ac.in</t>
+          <t>bhupali@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>arpitdwivedi1994@csjmu.ac.in</t>
+          <t>bijan@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>arunkgupta@csjmu.ac.in</t>
+          <t>bijan@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>arvindchauhan@csjmu.ac.in</t>
+          <t>bijitchoudhuri@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ashokkumarllm@csjmu.ac.in</t>
+          <t>biken@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>atulagnitotri@csjmu.ac.in</t>
+          <t>binita@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>awanish@csjmu.ac.in</t>
+          <t>binotipatro@mba.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>badrinarayanmishra@csjmu.ac.in</t>
+          <t>bipul@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>bappamaji@csjmu.ac.in</t>
+          <t>bishmitabhatacharjee31@gmail.com</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>bhanupratapsingh@csjmu.ac.in</t>
+          <t>biswajitsahoo@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>bhoomikayadav@csjmu.ac.in</t>
+          <t>bkr@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>bpsingh@csjmu.ac.in</t>
+          <t>bnghosh@che.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>brijendra@csjmu.ac.in</t>
+          <t>bpd@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>brishtimitra@csjmu.ac.in</t>
+          <t>bssil@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>cdoehelpline@csjmu.ac.in</t>
+          <t>chandrajit@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>chandrasekhar@csjmu.ac.in</t>
+          <t>chayan@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>chandreshsharma@csjmu.ac.in</t>
+          <t>chukhu@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>charukhan@csjmu.ac.in</t>
+          <t>cksahoo@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>chauhan10031981@csjmu.ac.in</t>
+          <t>d.rahul273@gmail.com</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>dakforanshu@gmail.com</t>
+          <t>dalton@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>deepak@csjmu.ac.in</t>
+          <t>dchowdhury@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>deepmalanigam@csjmu.ac.in</t>
+          <t>debabratabarman1967@gmail.com</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>dheeraj@csjmu.ac.in</t>
+          <t>debasish@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>digvijaysharma@csjmu.ac.in</t>
+          <t>debayan@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>diksha@csjmu.ac.in</t>
+          <t>debjit@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>dipeshverma@csjmu.ac.in</t>
+          <t>debtanay@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>divyanshshukla@csjmu.ac.in</t>
+          <t>deepanjal@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>dksingh@csjmu.ac.in</t>
+          <t>dibakar@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>dphysicaleducation@csjmu.ac.in</t>
+          <t>dibya@mba.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>drankittrivedi@csjmu.ac.in</t>
+          <t>dillip@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>drdhananjaydey@csjmu.ac.in</t>
+          <t>dinamanibiswal@hum.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>drdiwakarawasthi@gmail.com</t>
+          <t>dinesh@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>drmanasupadhyay@csjmu.ac.in</t>
+          <t>dipanjan@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>drmohitkumar@csjmu.ac.in</t>
+          <t>dipankar@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>drouptiyadav@csjmu.ac.in</t>
+          <t>dipjyoti@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>drpankajdwivedi.law@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>drpnpathak@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>drpoojaagarwal@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>drprabhatgauravmishra@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/hi/home</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>drprabhatkdwivedi@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/contact-us</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>drpramodkumar@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/academic/academic-contact</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>drprashant@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/ph-d-admission-for-january-to-june-2026-session</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>drprashanttrivedi@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/admission-details/active-studentcorner</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>drpravinagrawal@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/admission-details/admission-intake-status</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>drrahultiwari@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/mba-admission-2026-28</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>drrajeevmishra@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/ccmn-jam-admission</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>drramkishore@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/admission-details/scholarship-details</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>drrichamishra@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/screen-reader-access</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>drrichashukla@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/admission-details/archive-studentcorner</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>drroleesharma@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/courses/m-tech-m-sc-admission</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>drsandeepkporwal@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/admission-details/admission-notices</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>drsanjeevksingh@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/courses/ph-d-admission</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>drsaravankumaryadav@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/courses/m-b-a-admission</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>drsharaddixit@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/dasa-admission-2023</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>drshashikanttripathi@csjmu.ac.in</t>
+          <t>director@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/courses/b-tech-admission</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>drsnehpandey@csjmu.ac.in</t>
+          <t>djbora@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>drsonalimaurya@csjmu.ac.in</t>
+          <t>dkbaidya@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>drsonigupta@csjmu.ac.in</t>
+          <t>doren@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>drsurendrakumar@csjmu.ac.in</t>
+          <t>dristd_st@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>drvimalsingh@csjmu.ac.in</t>
+          <t>dsgurjar@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>e1229@csjmu.ac.in</t>
+          <t>dulal@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ektakhare@csjmu.ac.in</t>
+          <t>fazal@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>gauravkumar@csjmu.ac.in</t>
+          <t>gantidma@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>gauribhadauria@csjmu.ac.in</t>
+          <t>gaurav@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>gopal@csjmu.ac.in</t>
+          <t>gautamchoubey@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>guest119@csjmu.ac.in</t>
+          <t>gpkeshri@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>gyanendrasingh@csjmu.ac.in</t>
+          <t>guddus_stf@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>hemantkumar@csjmu.ac.in</t>
+          <t>harishore@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>himanshu@csjmu.ac.in</t>
+          <t>himadrid_st@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>himanshushukla@csjmu.ac.in</t>
+          <t>himanshu@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>hinavaish@csjmu.ac.in</t>
+          <t>jayshree@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>hradesh@csjmu.ac.in</t>
+          <t>jpmishra@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>hrishabh@csjmu.ac.in</t>
+          <t>jupitara@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>indreshs@csjmu.ac.in</t>
+          <t>juthika@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>info@csjmu.ac.in</t>
+          <t>jyotirmoy@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>izharalikhan@csjmu.ac.in</t>
+          <t>kalyan@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>jainrahul@csjmu.ac.in</t>
+          <t>kavicharan@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>jainsumit@csjmu.ac.in</t>
+          <t>kedarnath@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>jitendradobral@csjmu.ac.in</t>
+          <t>klb@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>jrgayen@gmail.com</t>
+          <t>koena@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>juitbali@csjmu.ac.in</t>
+          <t>koushik@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>jyoti@csjmu.ac.in</t>
+          <t>ktaimoor@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>kalpanakushwaha@csjmu.ac.in</t>
+          <t>kulkarni@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>kalpnaagnihotri@csjmu.ac.in</t>
+          <t>kumarnits@yahoo.com</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>kamalkant@csjmu.ac.in</t>
+          <t>lakshman@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>kaushikitrivedi@csjmu.ac.in</t>
+          <t>lcsaikia@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>kcjain@csjmu.ac.in</t>
+          <t>ldsingh@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>kiranjha@csjmu.ac.in</t>
+          <t>lintu@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>kirankky15j98@gmail.com</t>
+          <t>m123nath@gmail.com</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>kkchauhan@csjmu.ac.in</t>
+          <t>maa@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>laxmankumar@csjmu.ac.in</t>
+          <t>malayaduttaborah@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>madhulikasingh@csjmu.ac.in</t>
+          <t>mallikarjuna@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>mamta@csjmu.ac.in</t>
+          <t>maqbul@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>mamtasagar@csjmu.ac.in</t>
+          <t>mausumi@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>mamtatiwari@csjmu.ac.in</t>
+          <t>mazaman@che.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>mamtatiwaripharmaceutical@csjmu.ac.in</t>
+          <t>mdiwakar@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>manasibajpai@csjmu.ac.in</t>
+          <t>mita@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>manishitripathi15@csjmu.ac.in</t>
+          <t>mlvprasad@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>manishmaster99@gmail.com</t>
+          <t>monowar@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>manojkumar@csjmu.ac.in</t>
+          <t>munmun@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>mayankjindal@csjmu.ac.in</t>
+          <t>murugan.rmn@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>mayurisinghllm@csjmu.ac.in</t>
+          <t>nabanita@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>mayurrahul@csjmu.ac.in</t>
+          <t>nalin@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>meenakshigupta@csjmu.ac.in</t>
+          <t>naresh_stf@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>meghnabajpai@csjmu.ac.in</t>
+          <t>nbsingh@hum.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>mithaeewala@csjmu.ac.in</t>
+          <t>neeldeep@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>mohdmeerajsiddiqui@csjmu.ac.in</t>
+          <t>neha@hum.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>mohitawasthi@csjmu.ac.in</t>
+          <t>nidulsinha@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>mriduleshsingh@csjmu.ac.in</t>
+          <t>niharendu.dhar@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>mukeshranga@csjmu.ac.in</t>
+          <t>nilanjan@che.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>mukeshverma@csjmu.ac.in</t>
+          <t>nirmalendu@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>munishrastogi@csjmu.ac.in</t>
+          <t>nirmali@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>najmishabbir@csjmu.ac.in</t>
+          <t>nitesh@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>namitatiwari@csjmu.ac.in</t>
+          <t>noboraj@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>neerjasrivastava@csjmu.ac.in</t>
+          <t>nsmoyon@che.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>nehamishra@csjmu.ac.in</t>
+          <t>ojing@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>nehashukla@csjmu.ac.in</t>
+          <t>olympa@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>nimishasingh@csjmu.ac.in</t>
+          <t>pallab@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>nimishasinghkushwaha@csjmu.ac.in</t>
+          <t>panchali@hum.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>nirajkumar@csjmu.ac.in</t>
+          <t>pankaj@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>nishasharma@csjmu.ac.in</t>
+          <t>pankaj@phy.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>niyatipadhi@csjmu.ac.in</t>
+          <t>pantha@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>nks@csjmu.ac.in</t>
+          <t>papri@che.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>omkar@csjmu.ac.in</t>
+          <t>paramita@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>ompal@csjmu.ac.in</t>
+          <t>parbin@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>omshankargupta@csjmu.ac.in</t>
+          <t>parikshit@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>pallavimishra@csjmu.ac.in</t>
+          <t>partha@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>pallavitiwari@csjmu.ac.in</t>
+          <t>partha@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>parulawasthi@csjmu.ac.in</t>
+          <t>partha@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>pawan@csjmu.ac.in</t>
+          <t>partha@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>pbpatel@csjmu.ac.in</t>
+          <t>parthajit@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>poojasingh@csjmu.ac.in</t>
+          <t>parthasarathi@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>poonamdixit@csjmu.ac.in</t>
+          <t>pdebroy@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>prabalpratapsingh@csjmu.ac.in</t>
+          <t>pijusde@rediffmail.com</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>prabhakarpandey@csjmu.ac.in</t>
+          <t>pinki@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>prabhatsingh@csjmu.ac.in</t>
+          <t>pitambar@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>pradeeprajput@csjmu.ac.in</t>
+          <t>pmondal@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>prakashchandragupta@csjmu.ac.in</t>
+          <t>ppatowari@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>prakashnarainpandey@csjmu.ac.in</t>
+          <t>prabina@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>prashantsingh@csjmu.ac.in</t>
+          <t>pranjit@che.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>prashantsrivastava@csjmu.ac.in</t>
+          <t>prasanta@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>prateekagarwal@csjmu.ac.in</t>
+          <t>prashanth@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>prateeksrivastava@csjmu.ac.in</t>
+          <t>praveen@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>pratimakatiyar@csjmu.ac.in</t>
+          <t>prosun@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>praveenkatiyar@csjmu.ac.in</t>
+          <t>psneog@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>preetisingh@csjmu.ac.in</t>
+          <t>pulak.nath@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>priyaawasthi@csjmu.ac.in</t>
+          <t>purushottam@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>priyanka@csjmu.ac.in</t>
+          <t>puspa.devi@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>priyankashukla@csjmu.ac.in</t>
+          <t>rajarshi@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>priyatiwari@csjmu.ac.in</t>
+          <t>rajdeep@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>pulatsyashukla@csjmu.ac.in</t>
+          <t>rajeeb@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>purushottamsinghniranjan@csjmu.ac.in</t>
+          <t>rajeev@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>pushpamamoria@csjmu.ac.in</t>
+          <t>rajesh@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>rabins@csjmu.ac.in</t>
+          <t>rajib.kahar@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>raghwendra@csjmu.ac.in</t>
+          <t>rajkumar@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>raginiswarnkar@csjmu.ac.in</t>
+          <t>raju@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>rahulagarwal@csjmu.ac.in</t>
+          <t>ram@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>raj@csjmu.ac.in</t>
+          <t>ramakrishna@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>rajesh@csjmu.ac.in</t>
+          <t>ramanujam@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>rajeshkumar@csjmu.ac.in</t>
+          <t>ramkondasani@mba.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>rakeshsharma@csjmu.ac.in</t>
+          <t>ranjay@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>ramendra@csjmu.ac.in</t>
+          <t>rdmisra@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>ramjanma@csjmu.ac.in</t>
+          <t>reena@hum.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>ramnayan@csjmu.ac.in</t>
+          <t>registrar@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/contact-us</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>ranbirmukhya@csjmu.ac.in</t>
+          <t>rgnair@phy.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>ranjanagautam@csjmu.ac.in</t>
+          <t>rgnair@phy.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/ccmn-jam-admission</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>rashmidubey@csjmu.ac.in</t>
+          <t>rhlaskar@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/ccmn-jam-admission</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>rashmigautam@csjmu.ac.in</t>
+          <t>rhlaskar@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>rashmigore@csjmu.ac.in</t>
+          <t>rimmin_stf@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>ratnartuh@csjmu.ac.in</t>
+          <t>ripon@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>ratnartuh@gmail.com</t>
+          <t>risha@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>ratnashukla@csjmu.ac.in</t>
+          <t>rokhum@che.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>ravikantmishra@csjmu.ac.in</t>
+          <t>roopjyotideb@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>richaverma@csjmu.ac.in</t>
+          <t>rsingha_st@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>rishisrivastava@csjmu.ac.in</t>
+          <t>ruma@che.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>riteshagarwal@csjmu.ac.in</t>
+          <t>rupak@phy.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>rohitpanday@csjmu.ac.in</t>
+          <t>saheli@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>roopkishor@csjmu.ac.in</t>
+          <t>samir@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>rpsaini@csjmu.ac.in</t>
+          <t>santan@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>rvsls@csjmu.ac.in</t>
+          <t>santanu@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>sachinsharma@csjmu.ac.in</t>
+          <t>saroj@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>sachivgautam@csjmu.ac.in</t>
+          <t>saumya@phy.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>sacsjmu@gmail.com</t>
+          <t>saurabh@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>sajaysingh@csjmu.ac.in</t>
+          <t>saurabhverma@mba.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>samarendrchauhanllm@csjmu.ac.in</t>
+          <t>sb@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>samiuddin@csjmu.ac.in</t>
+          <t>seban@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>sandeep@csjmu.ac.in</t>
+          <t>shalder@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>sandesh@csjmu.ac.in</t>
+          <t>shankar@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>sanjeet@csjmu.ac.in</t>
+          <t>shanti@che.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>santoshkumaryadav@csjmu.ac.in</t>
+          <t>shashi@hum.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>sarveshmanitripathi@csjmu.ac.in</t>
+          <t>shlaskar@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>satyaprakashverma@csjmu.ac.in</t>
+          <t>shubham@mba.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>satyendrachauhan@csjmu.ac.in</t>
+          <t>shubhamdos3@gmail.com</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>saurabhtiwari@csjmu.ac.in</t>
+          <t>shuprajhaa@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>saurabhtripathi@csjmu.ac.in</t>
+          <t>simanchal@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>scpatel@csjmu.ac.in</t>
+          <t>sinha.bipon@gmail.com</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>shahalam@csjmu.ac.in</t>
+          <t>skpandey@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>shalinishukla@csjmu.ac.in</t>
+          <t>sksahoo@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>shashikmishra@csjmu.ac.in</t>
+          <t>sktripathy@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>shashwatkatiyar8@gmail.com</t>
+          <t>snehasish@phy.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>shashwatkatiyar@csjmu.ac.in</t>
+          <t>soma@mba.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>shekharverma@csjmu.ac.in</t>
+          <t>somnath@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>sheshmani@csjmu.ac.in</t>
+          <t>spal@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>shikhashukla@csjmu.ac.in</t>
+          <t>sreejith@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>shilpakaistha@csjmu.ac.in</t>
+          <t>sreenu@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>shilpidubey@csjmu.ac.in</t>
+          <t>srinivasan@phy.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>shilpikukreja@csjmu.ac.in</t>
+          <t>srmaity@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>shishupalsingh@csjmu.ac.in</t>
+          <t>ssd@che.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>shivansusachan@csjmu.ac.in</t>
+          <t>subhadeep@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>shivneet@csjmu.ac.in</t>
+          <t>subhadip@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>shobhit@csjmu.ac.in</t>
+          <t>subhajit@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>shreyasingh@csjmu.ac.in</t>
+          <t>subhasis@phy.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>shriprakash747@gmail.com</t>
+          <t>subhradeep.dhar@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>shubhambajpai@csjmu.ac.in</t>
+          <t>subhrajit.dutta@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>shubhamswarnkar@csjmu.ac.in</t>
+          <t>subrat@phy.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>shubhendra@csjmu.ac.in</t>
+          <t>subrata@math.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>shweta@csjmu.ac.in</t>
+          <t>sucharita@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>sidhanshurai@csjmu.ac.in</t>
+          <t>sudarsan@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>skawasthi@csjmu.ac.in</t>
+          <t>sudip@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>smitagupta@csjmu.ac.in</t>
+          <t>sudipk_st@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>smritiroyllm@csjmu.ac.in</t>
+          <t>sudipta@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>so.maths@csjmu.ac.in</t>
+          <t>suganya@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>somesh@csjmu.ac.in</t>
+          <t>sujitnath@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>sonamgupta@csjmu.ac.in</t>
+          <t>sujupat@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>ssc@csjmu.ac.in</t>
+          <t>sukumar@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>sudesh@csjmu.ac.in</t>
+          <t>sumallya@hum.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>sudhanshu@csjmu.ac.in</t>
+          <t>sumanc_stf@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>sudhir@csjmu.ac.in</t>
+          <t>sumit@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>sudhirverma@csjmu.ac.in</t>
+          <t>sumita@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>sumanbiswas@csjmu.ac.in</t>
+          <t>sumitra@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>sunilkumar@csjmu.ac.in</t>
+          <t>sunil@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>suruchi@csjmu.ac.in</t>
+          <t>sunilkumar@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>swarnakshiupadhyay@csjmu.ac.in</t>
+          <t>suprava@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>swatisrivastava@csjmu.ac.in</t>
+          <t>surajs_st@nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>tanisha@csjmu.ac.in</t>
+          <t>surush18@gmail.com</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/Administration/officers-and-staffs</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>tanuja@csjmu.ac.in</t>
+          <t>sushant@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>ucsharma@csjmu.ac.in</t>
+          <t>susmita@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>umesh@csjmu.ac.in</t>
+          <t>susmita@phy.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>urvashi@csjmu.ac.in</t>
+          <t>swapna@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>vaibhavsaxena@csjmu.ac.in</t>
+          <t>swati@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>varsha@csjmu.ac.in</t>
+          <t>tanayanayak@mba.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>varshagupta@csjmu.ac.in</t>
+          <t>tanmoy@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>vershaprasad@csjmu.ac.in</t>
+          <t>tapan_pradhan@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>vijaykashyap@csjmu.ac.in</t>
+          <t>tauhidr@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>vikashkatiyar@csjmu.ac.in</t>
+          <t>triptigoel@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>vinaysingh@csjmu.ac.in</t>
+          <t>trlenka@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>vineetasingh@csjmu.ac.in</t>
+          <t>ujjal@ece.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>vinita@csjmu.ac.in</t>
+          <t>ujjal@hum.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>vinod@csjmu.ac.in</t>
+          <t>ujwala@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>vishalawasthi@csjmu.ac.in</t>
+          <t>umakanta@cse.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>vishalchand@csjmu.ac.in</t>
+          <t>upendra@civil.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>vishalsharma@csjmu.ac.in</t>
+          <t>vinyas@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>vishwdeepmishra@csjmu.ac.in</t>
+          <t>vipin@ei.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>viveksinghsachan@csjmu.ac.in</t>
+          <t>vivekanandan@ee.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>vkcontinentalexports@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" t="inlineStr">
-        <is>
-          <t>vksachan@csjmu.ac.in</t>
-        </is>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="inlineStr">
-        <is>
-          <t>vkyadav@csjmu.ac.in</t>
-        </is>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="inlineStr">
-        <is>
-          <t>warshisingh@csjmu.ac.in</t>
-        </is>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="inlineStr">
-        <is>
-          <t>yastuti@csjmu.ac.in</t>
-        </is>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" t="inlineStr">
-        <is>
-          <t>yogendrakumarpandey@csjmu.ac.in</t>
-        </is>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="inlineStr">
-        <is>
-          <t>yogeshchndra@csjmu.ac.in</t>
-        </is>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="inlineStr">
-        <is>
-          <t>ypramod@csjmu.ac.in</t>
+          <t>yogesh@mech.nits.ac.in</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>https://www.nits.ac.in/more/faculty-list</t>
         </is>
       </c>
     </row>

</xml_diff>